<commit_message>
test/excel: Excel for Mac on lines/files (second run) and lines/held, as predicted but where Excel merges the styles of a row and a column it formats across each other; the round-trip books styles, hidden and struct-styles-styled sent again (the writer writes the cells where lines cross) and read back as written; the fit cases colformat sent again: Excel shows the column's format, the known difference writer goes (ru-RU colformat-2 shows the Mac's lower-case month, macRegional)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/lines/files/typed-crossing.xlsx
+++ b/test/excel/lines/files/typed-crossing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-30511/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-91180/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{605FE4E7-1B53-AC41-A2A3-8B1DDB496D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{633D7ABE-DEE6-CA41-AB9A-1A19403137EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>